<commit_message>
updates to param sync and point layout tools
</commit_message>
<xml_diff>
--- a/MC Tools.tab/Utilities.panel/Exports.pulldown/GenerateBulkBOM.pushbutton/MR-BOM.xlsx
+++ b/MC Tools.tab/Utilities.panel/Exports.pulldown/GenerateBulkBOM.pushbutton/MR-BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Egnyte\Shared\BIM\Murray CADetailing Dept\REVIT\MURRAY RIBBON\Murray.extension\MurrayTools.tab\Utilities.panel\ProjectUtilities.Stack\Exports.pulldown\GenerateBulkBOM.pushbutton\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Egnyte\Shared\BIM\Murray CADetailing Dept\REVIT\MURRAY RIBBON\Murray.extension\MC Tools.tab\Utilities.panel\Exports.pulldown\GenerateBulkBOM.pushbutton\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5616BDA3-DD21-4F48-8BF2-18EEF87BDE3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{160B2967-97BA-4E8C-A1A3-BD93652CACAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="3900" windowWidth="28800" windowHeight="15345" xr2:uid="{3AEB8DE0-985F-4A48-8335-FFD4EE2C061B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{3AEB8DE0-985F-4A48-8335-FFD4EE2C061B}"/>
   </bookViews>
   <sheets>
     <sheet name="MEP Fabrication Pipe BOM" sheetId="1" r:id="rId1"/>
@@ -38,10 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
-    <t>18414  South  Santa  Fe  Avenue Rancho  Dominguez,  CA  90221
-Phone:  (310)  637-1500        Fax:  (310)  637-2819</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="9.5"/>
@@ -390,6 +386,10 @@
   </si>
   <si>
     <t>BOM DESCRIPTION HERE</t>
+  </si>
+  <si>
+    <t>5995 Plaza Drive Cypress, CA 90630
+Phone:  (310)  637-1500        Fax:  (310)  637-2819</t>
   </si>
 </sst>
 </file>
@@ -674,12 +674,60 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -689,6 +737,18 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -712,66 +772,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1173,204 +1173,204 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="18"/>
+      <c r="G1" s="19"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="15"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="20"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="15"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="23"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="15"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="25"/>
-      <c r="G1" s="36"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="33"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="37"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="33"/>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="39"/>
-      <c r="G3" s="40"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="33"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="24"/>
+      <c r="G4" s="25"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="15"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="11"/>
-      <c r="G4" s="12"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="33"/>
-      <c r="B5" s="34"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="43" t="s">
+      <c r="F5" s="24"/>
+      <c r="G5" s="25"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="15"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="11"/>
-      <c r="G5" s="12"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="33"/>
-      <c r="B6" s="34"/>
-      <c r="C6" s="34"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="43" t="s">
+      <c r="F6" s="24"/>
+      <c r="G6" s="25"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="11"/>
-      <c r="G6" s="12"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="33"/>
-      <c r="B7" s="34"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="7" t="s">
+      <c r="F7" s="26">
+        <f ca="1">NOW()</f>
+        <v>46196.447998958334</v>
+      </c>
+      <c r="G7" s="27"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="29"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="24"/>
+      <c r="G8" s="25"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="29"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="41">
-        <f ca="1">NOW()</f>
-        <v>45797.43305659722</v>
-      </c>
-      <c r="G7" s="42"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="8" t="s">
+      <c r="F9" s="32"/>
+      <c r="G9" s="33"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="29"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="24"/>
+      <c r="G10" s="25"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="29"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="24"/>
+      <c r="G11" s="25"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="24"/>
+      <c r="G12" s="25"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="38" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="39"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="24"/>
+      <c r="G13" s="25"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="42"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="24"/>
+      <c r="G14" s="25"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="11"/>
-      <c r="G8" s="12"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="27"/>
-      <c r="G9" s="28"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="11"/>
-      <c r="G10" s="12"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11" s="11"/>
-      <c r="G11" s="12"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" s="11"/>
-      <c r="G12" s="12"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="11"/>
-      <c r="G13" s="12"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="5" t="s">
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="11"/>
-      <c r="G14" s="12"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="16"/>
-      <c r="G15" s="17"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="37"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
@@ -1378,6 +1378,22 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="A1:D7"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="E2:G2"/>
@@ -1386,22 +1402,6 @@
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="E5:G5"/>
     <mergeCell ref="E6:G6"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A14:C14"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>